<commit_message>
Replace body masking with equipment fit tuning
Add workbook-authored fit_scale/fit_offset on equipment visual mappings and
bake subtle per-piece bind-pose inflation into skinned armor GLBs. Skinned
overlays keep runtime transforms unchanged so skeleton rebinding and CG5 morph
sync stay intact; rigid items may compose fit at resolve time when authored.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -8954,7 +8954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9023,6 +9023,16 @@
           <t>Consumed Morph Params</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Fit Scale</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Fit Offset</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9060,7 +9070,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9098,7 +9107,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9136,7 +9144,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9174,7 +9181,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9227,7 +9233,6 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9280,7 +9285,6 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9318,7 +9322,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9356,7 +9359,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9394,7 +9396,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9432,7 +9433,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9470,7 +9470,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9508,7 +9507,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9546,7 +9544,6 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9584,7 +9581,6 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9622,7 +9618,6 @@
           <t>0,1,0,0</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9660,7 +9655,6 @@
           <t>0,1,0,0</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9688,6 +9682,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9715,6 +9715,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9742,6 +9748,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>1.035</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9769,6 +9781,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>1.035</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9796,6 +9814,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9823,6 +9847,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9845,7 +9875,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9868,7 +9897,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9896,6 +9924,16 @@
           <t>head_size</t>
         </is>
       </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0,0.004,0</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9923,6 +9961,16 @@
           <t>head_size</t>
         </is>
       </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0,0.004,0</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9950,6 +9998,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9977,6 +10031,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10004,6 +10064,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>1.035</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10031,6 +10097,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>1.035</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10058,6 +10130,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10085,6 +10163,12 @@
           <t>build,fat,muscle</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10107,7 +10191,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10130,7 +10213,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add regional human body morph targets
Author CG9 regional morph deltas on male/female human GLBs, extend workbook mappings, and validate the full human morph vocabulary.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -9687,7 +9687,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9720,7 +9719,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9753,7 +9751,6 @@
           <t>1.035</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9786,7 +9783,6 @@
           <t>1.035</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9819,7 +9815,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9852,7 +9847,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10003,7 +9997,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10036,7 +10029,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10069,7 +10061,6 @@
           <t>1.035</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10102,7 +10093,6 @@
           <t>1.035</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10135,7 +10125,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10168,7 +10157,6 @@
           <t>1.04</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10812,7 +10800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11070,17 +11058,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>shoulders</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>build_broad</t>
+          <t>shoulders_broad</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -11105,17 +11093,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>shoulders</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>build_narrow</t>
+          <t>shoulders_narrow</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -11140,17 +11128,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>fat</t>
+          <t>torso</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>fat_soft</t>
+          <t>torso_broad</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -11175,22 +11163,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>muscle</t>
+          <t>torso</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>muscle_define</t>
+          <t>torso_narrow</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Above Default</t>
+          <t>Below Default</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -11210,17 +11198,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>head_size</t>
+          <t>arms</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>head_large</t>
+          <t>arms_thick</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -11245,17 +11233,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>human_female</t>
+          <t>human_male</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>head_size</t>
+          <t>arms</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>head_small</t>
+          <t>arms_thin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -11267,6 +11255,706 @@
         <v>1</v>
       </c>
       <c r="G13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>human_male</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>hips</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>hips_broad</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>human_male</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>hips</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>hips_narrow</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>human_male</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>legs_thick</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>human_male</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>legs_thin</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>build_broad</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>build</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>build_narrow</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>fat</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>fat_soft</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>muscle</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>muscle_define</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>head_size</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>head_large</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>head_size</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>head_small</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>shoulders</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>shoulders_broad</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>shoulders</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>shoulders_narrow</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>torso_broad</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>torso</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>torso_narrow</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>arms</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>arms_thick</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>arms</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>arms_thin</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>hips</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>hips_broad</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>hips</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>hips_narrow</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>legs_thick</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Above Default</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>human</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>human_female</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>legs_thin</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Below Default</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
Add regional equipment morph targets
Extend CG5 equipment morph authoring and workbook consumption so skinned clothing follows regional body sliders via the existing transfer pipeline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -9070,6 +9070,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9107,6 +9108,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9144,6 +9146,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9181,6 +9184,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9233,6 +9237,7 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9285,6 +9290,7 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9322,6 +9328,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9359,6 +9366,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9396,6 +9404,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9433,6 +9442,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9470,6 +9480,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9507,6 +9518,7 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9544,6 +9556,7 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9581,6 +9594,7 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9618,6 +9632,7 @@
           <t>0,1,0,0</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9655,6 +9670,7 @@
           <t>0,1,0,0</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9679,7 +9695,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,shoulders,torso,hips</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -9711,7 +9727,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,shoulders,torso,hips</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -9743,7 +9759,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,arms</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -9775,7 +9791,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,arms</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -9807,7 +9823,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,legs,hips</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -9839,7 +9855,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,legs,hips</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -9869,6 +9885,7 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9891,6 +9908,7 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9989,7 +10007,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,shoulders,torso,hips</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -10021,7 +10039,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,shoulders,torso,hips</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -10053,7 +10071,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,arms</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -10085,7 +10103,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,arms</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -10117,7 +10135,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,legs,hips</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -10149,7 +10167,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>build,fat,muscle</t>
+          <t>build,fat,muscle,legs,hips</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -10179,6 +10197,7 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10201,6 +10220,7 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Import 14 Monsters Full Pack units as GLBs and workbook rows.
Adds Blender batch pipeline, U-0006 through U-0019 with animation profiles and weapons. Documents 15 SK-FBX import failures for follow-up.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -2105,7 +2105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16.85546875" bestFit="1" customWidth="1" style="36" min="1" max="1"/>
@@ -2868,6 +2868,804 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>weapon_tyranopode_primary</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tyranopode Attack</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>JumpTentaclesSmashAttack</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>weapon_muscomorph_primary</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Muscomorph Attack</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>BiteAttack</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>weapon_telluropod_primary</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Telluropod Attack</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>BiteAttack</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>weapon_clypeosaurus_primary</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Clypeosaurus Attack</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>RoarAntennaElectricAttack</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>weapon_giant_slug_primary</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Giant Slug Attack</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CrawlForwardTurnLeftSpittersAttack</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>weapon_karcinomorph_primary</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Karcinomorph Attack</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>JumpLegsAttack</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>weapon_scyver_primary</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Scyver Attack</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>BiteAttack1</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>weapon_scolomorph_primary</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Scolomorph Attack</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>BiteForwardAttack</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>weapon_tetrachnide_primary</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Tetrachnide Attack</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>ClawsAttack</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>weapon_vespomorph_primary</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Vespomorph Attack</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>FlyBiteAttack</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>weapon_morphorrid_primary</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Morphorrid Attack</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>JumpTentaclesAttack</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>weapon_carcidonte_primary</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Carcidonte Attack</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>ClawsAttack</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>weapon_entomorane_primary</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Entomorane Attack</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>BiteAttack</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>weapon_laminferox_primary</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Laminferox Attack</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Intrinsic monster attack (placeholder balance).</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>6</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Slashing</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Melee</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>BiteAttack</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Enemies, Wildlife</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2879,7 +3677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3144,6 +3942,632 @@
           <t>Mine</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tyranopode</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>GetHit</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CrawlLeft</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>CrawlRight</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>muscomorph</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>GetHit1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>CrawlLeft</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>CrawlRight</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>telluropod</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>clypeosaurus</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>TurnLeft</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>TurnRight</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>giant_slug</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>karcinomorph</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CrawlLeft</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>CrawlRight</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>scyver</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>scolomorph</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>tetrachnide</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CrawlForward</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>CrawlLeft</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CrawlRight</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>vespomorph</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>GetHit</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>morphorrid</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>carcidonte</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>entomorane</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Idle</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>laminferox</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>IdleBreathe</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>WalkForward</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4100,7 +5524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4203,6 +5627,244 @@
         </is>
       </c>
       <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tyranopode</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tyranopode</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>muscomorph</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Muscomorph</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>telluropod</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Telluropod</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>clypeosaurus</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Clypeosaurus</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>giant_slug</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Giant Slug</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>karcinomorph</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Karcinomorph</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>scyver</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Scyver</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>scolomorph</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Scolomorph</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>tetrachnide</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tetrachnide</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>vespomorph</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vespomorph</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>morphorrid</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Morphorrid</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>carcidonte</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Carcidonte</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>entomorane</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Entomorane</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>laminferox</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Laminferox</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -9070,7 +10732,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9108,7 +10769,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9146,7 +10806,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9184,7 +10843,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9237,7 +10895,6 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9290,7 +10947,6 @@
           <t>0.0,0.707,0.0,0.707</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9328,7 +10984,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9366,7 +11021,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9404,7 +11058,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9442,7 +11095,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9480,7 +11132,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9518,7 +11169,6 @@
           <t>0,-0.5,-0.5,0.5</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9556,7 +11206,6 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9594,7 +11243,6 @@
           <t>0.5,0.5,0.5,0.5</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9632,7 +11280,6 @@
           <t>0,1,0,0</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9670,7 +11317,6 @@
           <t>0,1,0,0</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9885,7 +11531,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9908,7 +11553,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10197,7 +11841,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -10220,7 +11863,6 @@
           <t>SkinnedOverlay</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12879,46 +14521,1334 @@
       </c>
     </row>
     <row r="7">
-      <c r="P7" s="11" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>U-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tyranopode</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>tyranopode</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>assets\units\tyranopode.glb</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H7" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="n">
+        <v>28</v>
+      </c>
+      <c r="O7" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P7" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="n">
+        <v>45</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>tyranopode</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>weapon_tyranopode_primary</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="8">
-      <c r="P8" s="11" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>U-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Muscomorph</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>muscomorph</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>assets\units\muscomorph.glb</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H8" t="n">
+        <v>7</v>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="n">
+        <v>28</v>
+      </c>
+      <c r="O8" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P8" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="n">
+        <v>45</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>muscomorph</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>weapon_muscomorph_primary</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="9">
-      <c r="P9" s="11" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>U-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Telluropod</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>telluropod</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>assets\units\telluropod.glb</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>40</v>
+      </c>
+      <c r="H9" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" t="n">
+        <v>28</v>
+      </c>
+      <c r="O9" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P9" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>45</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>telluropod</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>weapon_telluropod_primary</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="10">
-      <c r="P10" s="11" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>U-0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Clypeosaurus</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>clypeosaurus</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>assets\units\clypeosaurus.glb</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" t="n">
+        <v>2</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="n">
+        <v>28</v>
+      </c>
+      <c r="O10" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P10" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>45</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>clypeosaurus</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>weapon_clypeosaurus_primary</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="11">
-      <c r="P11" s="11" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>U-0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Giant Slug</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>giant_slug</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>assets\units\giant_slug.glb</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>40</v>
+      </c>
+      <c r="H11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" t="n">
+        <v>6</v>
+      </c>
+      <c r="J11" t="n">
+        <v>6</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="n">
+        <v>28</v>
+      </c>
+      <c r="O11" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P11" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>45</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>giant_slug</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>weapon_giant_slug_primary</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="12">
-      <c r="P12" s="11" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>U-0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Karcinomorph</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>karcinomorph</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>assets\units\karcinomorph.glb</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>40</v>
+      </c>
+      <c r="H12" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>6</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="n">
+        <v>2</v>
+      </c>
+      <c r="N12" t="n">
+        <v>28</v>
+      </c>
+      <c r="O12" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P12" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>45</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>karcinomorph</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>weapon_karcinomorph_primary</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="13">
-      <c r="P13" s="11" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>U-0012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Scyver</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>scyver</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>assets\units\scyver.glb</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>40</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7</v>
+      </c>
+      <c r="I13" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>28</v>
+      </c>
+      <c r="O13" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P13" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>45</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>scyver</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>weapon_scyver_primary</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="14">
-      <c r="P14" s="11" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>U-0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Scolomorph</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>scolomorph</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>assets\units\scolomorph.glb</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" t="n">
+        <v>40</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N14" t="n">
+        <v>28</v>
+      </c>
+      <c r="O14" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P14" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>45</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>scolomorph</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>weapon_scolomorph_primary</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="15">
-      <c r="P15" s="11" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>U-0014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tetrachnide</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>tetrachnide</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>assets\units\tetrachnide.glb</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>40</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" t="n">
+        <v>6</v>
+      </c>
+      <c r="J15" t="n">
+        <v>6</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2</v>
+      </c>
+      <c r="N15" t="n">
+        <v>28</v>
+      </c>
+      <c r="O15" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P15" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="n">
+        <v>45</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>tetrachnide</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>weapon_tetrachnide_primary</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="16">
-      <c r="P16" s="11" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>U-0015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vespomorph</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>vespomorph</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>assets\units\vespomorph.glb</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" t="n">
+        <v>40</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2</v>
+      </c>
+      <c r="N16" t="n">
+        <v>28</v>
+      </c>
+      <c r="O16" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P16" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="n">
+        <v>45</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>vespomorph</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>weapon_vespomorph_primary</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="17">
-      <c r="P17" s="11" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>U-0016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Morphorrid</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>morphorrid</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>assets\units\morphorrid.glb</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>40</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6</v>
+      </c>
+      <c r="J17" t="n">
+        <v>6</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" t="n">
+        <v>2</v>
+      </c>
+      <c r="N17" t="n">
+        <v>28</v>
+      </c>
+      <c r="O17" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P17" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="n">
+        <v>45</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>morphorrid</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>weapon_morphorrid_primary</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="18">
-      <c r="P18" s="11" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>U-0017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Carcidonte</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>carcidonte</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>assets\units\carcidonte.glb</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>3</v>
+      </c>
+      <c r="G18" t="n">
+        <v>40</v>
+      </c>
+      <c r="H18" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" t="n">
+        <v>6</v>
+      </c>
+      <c r="K18" t="n">
+        <v>5</v>
+      </c>
+      <c r="L18" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N18" t="n">
+        <v>28</v>
+      </c>
+      <c r="O18" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P18" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" t="n">
+        <v>45</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>carcidonte</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>weapon_carcidonte_primary</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="19">
-      <c r="P19" s="11" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>U-0018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Entomorane</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>entomorane</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>assets\units\entomorane.glb</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H19" t="n">
+        <v>7</v>
+      </c>
+      <c r="I19" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2</v>
+      </c>
+      <c r="N19" t="n">
+        <v>28</v>
+      </c>
+      <c r="O19" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P19" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1</v>
+      </c>
+      <c r="S19" t="n">
+        <v>45</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>entomorane</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>weapon_entomorane_primary</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="20">
-      <c r="P20" s="11" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>U-0019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Laminferox</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>wild</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>laminferox</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>assets\units\laminferox.glb</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" t="n">
+        <v>40</v>
+      </c>
+      <c r="H20" t="n">
+        <v>7</v>
+      </c>
+      <c r="I20" t="n">
+        <v>6</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6</v>
+      </c>
+      <c r="K20" t="n">
+        <v>5</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" t="n">
+        <v>28</v>
+      </c>
+      <c r="O20" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P20" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>laminferox</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>weapon_laminferox_primary</t>
+        </is>
+      </c>
+      <c r="X20" t="n">
+        <v>180</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="21">
       <c r="P21" s="11" t="n"/>
@@ -12958,6 +15888,7 @@
       <c r="O28" s="10" t="n"/>
       <c r="P28" s="12" t="n"/>
     </row>
+    <row r="29"/>
     <row r="30" ht="15.75" customHeight="1" s="36">
       <c r="A30" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix bufomorph catalog import (species + stats) and unify muscomorph skin for runtime spikes.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -4594,7 +4594,6 @@
           <t>GetHitFront</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5551,7 +5550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5892,6 +5891,23 @@
         </is>
       </c>
       <c r="C19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>bufomorph</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Bufomorph</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -15903,7 +15919,40 @@
           <t>assets\units\bufomorph.glb</t>
         </is>
       </c>
+      <c r="F21" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" t="n">
+        <v>40</v>
+      </c>
+      <c r="H21" t="n">
+        <v>7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2</v>
+      </c>
       <c r="P21" s="11" t="n"/>
+      <c r="Q21" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="n">
+        <v>45</v>
+      </c>
       <c r="T21" t="inlineStr">
         <is>
           <t>bufomorph</t>
@@ -15921,6 +15970,12 @@
       </c>
       <c r="X21" t="n">
         <v>180</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>360</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Fix bufomorph unit import: set Power Rating, Total Stats, and Tier on U-0029.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Chasma Design.xlsx
+++ b/Chasma Design.xlsx
@@ -15943,7 +15943,17 @@
       <c r="M21" t="n">
         <v>2</v>
       </c>
-      <c r="P21" s="11" t="n"/>
+      <c r="N21" t="n">
+        <v>28</v>
+      </c>
+      <c r="O21" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="P21" s="11" t="inlineStr">
+        <is>
+          <t>Elite</t>
+        </is>
+      </c>
       <c r="Q21" t="n">
         <v>3.5</v>
       </c>

</xml_diff>